<commit_message>
fix: Dong bo 100% giua Script SQL va cac file Excel mau danh muc
</commit_message>
<xml_diff>
--- a/data/catalogs/pharmacy_mappings.xlsx
+++ b/data/catalogs/pharmacy_mappings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -521,7 +521,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Khoa Phụ Sản</t>
+          <t>Khoa Cấp cứu</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -538,32 +538,66 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Khoa Phẫu thuật - GMHS</t>
+          <t>Khoa Phụ Sản</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>KHO_GMHS</t>
+          <t>KHO_LE_NOITRU</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Kho Phẫu thuật - GMHS</t>
+          <t>Kho lẻ Nội trú</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>Khoa Phụ Sản</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>KHO_VTYT_NOITRU</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Kho vật tư Nội trú</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Khoa Phẫu thuật - GMHS</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>KHO_GMHS</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Kho Phẫu thuật - GMHS</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Khoa Xét Nghiệm</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>KHO_VTYT_XN</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Kho vật tư Xét nghiệm</t>
         </is>

</xml_diff>